<commit_message>
Update formal knowledge sources
</commit_message>
<xml_diff>
--- a/knowledge-source/DIC套餐功能支持表.xlsx
+++ b/knowledge-source/DIC套餐功能支持表.xlsx
@@ -67,13 +67,13 @@
     <t xml:space="preserve">Share+/共享版+</t>
   </si>
   <si>
-    <t xml:space="preserve">base plan price</t>
+    <t xml:space="preserve">plan price</t>
   </si>
   <si>
     <t xml:space="preserve">included profiles</t>
   </si>
   <si>
-    <t xml:space="preserve">additional profiles</t>
+    <t xml:space="preserve">additional profile pricing</t>
   </si>
   <si>
     <t xml:space="preserve">Not supported</t>
@@ -120,7 +120,7 @@
     <t xml:space="preserve">1 (includes Super Admin)</t>
   </si>
   <si>
-    <t xml:space="preserve">additional members</t>
+    <t xml:space="preserve">additional member pricing</t>
   </si>
   <si>
     <t xml:space="preserve">$3/month/member</t>
@@ -318,7 +318,7 @@
   <cellStyleXfs count="1">
     <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="false" applyNumberFormat="false" applyProtection="false" borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf applyAlignment="false" applyBorder="false" applyFill="false" applyFont="false" applyNumberFormat="false" applyProtection="false" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -336,6 +336,9 @@
     </xf>
     <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="true" applyProtection="false" borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0">
       <alignment vertical="center" wrapText="true"/>
@@ -661,12 +664,12 @@
     <outlinePr summaryBelow="false" summaryRight="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="18"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" max="1" min="1" style="0" width="29"/>
-    <col collapsed="false" customWidth="true" hidden="false" max="3" min="3" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" max="4" min="4" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" max="5" min="5" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" max="1" min="1" style="0" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" max="3" min="3" style="0" width="39"/>
+    <col collapsed="false" customWidth="true" hidden="false" max="4" min="4" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" max="5" min="5" style="0" width="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -686,7 +689,7 @@
         <v>5</v>
       </c>
     </row>
-    <row customHeight="true" ht="18" r="2">
+    <row customHeight="true" ht="16" r="2">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
@@ -703,8 +706,8 @@
         <v>138</v>
       </c>
     </row>
-    <row customHeight="true" ht="18" r="3">
-      <c r="A3" s="3" t="s">
+    <row customHeight="true" ht="16" r="3">
+      <c r="A3" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="4">
@@ -737,8 +740,8 @@
         <v>12</v>
       </c>
     </row>
-    <row customHeight="true" ht="132" r="5">
-      <c r="A5" s="6" t="s">
+    <row customHeight="true" ht="117" r="5">
+      <c r="A5" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="4">
@@ -754,8 +757,8 @@
         <v>14</v>
       </c>
     </row>
-    <row customHeight="true" ht="18" r="6">
-      <c r="A6" s="3" t="s">
+    <row customHeight="true" ht="16" r="6">
+      <c r="A6" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B6" s="4">
@@ -771,7 +774,7 @@
         <v>14</v>
       </c>
     </row>
-    <row customHeight="true" ht="18" r="7">
+    <row customHeight="true" ht="16" r="7">
       <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
@@ -788,8 +791,8 @@
         <v>14</v>
       </c>
     </row>
-    <row customHeight="true" ht="18" r="8">
-      <c r="A8" s="3" t="s">
+    <row customHeight="true" ht="16" r="8">
+      <c r="A8" s="6" t="s">
         <v>21</v>
       </c>
       <c r="B8" s="4" t="s">
@@ -805,8 +808,8 @@
         <v>9</v>
       </c>
     </row>
-    <row customHeight="true" ht="18" r="9">
-      <c r="A9" s="3" t="s">
+    <row customHeight="true" ht="16" r="9">
+      <c r="A9" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B9" s="4">
@@ -822,8 +825,8 @@
         <v>1</v>
       </c>
     </row>
-    <row customHeight="true" ht="18" r="10">
-      <c r="A10" s="3" t="s">
+    <row customHeight="true" ht="16" r="10">
+      <c r="A10" s="6" t="s">
         <v>25</v>
       </c>
       <c r="B10" s="4" t="s">
@@ -839,8 +842,8 @@
         <v>9</v>
       </c>
     </row>
-    <row customHeight="true" ht="18" r="11">
-      <c r="A11" s="3" t="s">
+    <row customHeight="true" ht="16" r="11">
+      <c r="A11" s="6" t="s">
         <v>27</v>
       </c>
       <c r="B11" s="4">
@@ -856,7 +859,7 @@
         <v>14</v>
       </c>
     </row>
-    <row customHeight="true" ht="18" r="12">
+    <row customHeight="true" ht="16" r="12">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -873,7 +876,7 @@
         <v>29</v>
       </c>
     </row>
-    <row customHeight="true" ht="18" r="13">
+    <row customHeight="true" ht="16" r="13">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -890,7 +893,7 @@
         <v>29</v>
       </c>
     </row>
-    <row customHeight="true" ht="18" r="14">
+    <row customHeight="true" ht="16" r="14">
       <c r="A14" t="s">
         <v>31</v>
       </c>
@@ -907,7 +910,7 @@
         <v>29</v>
       </c>
     </row>
-    <row customHeight="true" ht="18" r="15">
+    <row customHeight="true" ht="16" r="15">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -924,8 +927,8 @@
         <v>29</v>
       </c>
     </row>
-    <row customHeight="true" ht="18" r="16">
-      <c r="A16" s="3" t="s">
+    <row customHeight="true" ht="16" r="16">
+      <c r="A16" s="6" t="s">
         <v>33</v>
       </c>
       <c r="B16" s="4" t="s">
@@ -958,20 +961,20 @@
         <v>100</v>
       </c>
     </row>
-    <row customHeight="true" ht="18" r="18">
+    <row customHeight="true" ht="16" r="18">
       <c r="A18" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="7">
+      <c r="B18" s="8">
         <v>5</v>
       </c>
-      <c r="C18" s="7">
+      <c r="C18" s="8">
         <v>5</v>
       </c>
-      <c r="D18" s="7">
+      <c r="D18" s="8">
         <v>500</v>
       </c>
-      <c r="E18" s="7">
+      <c r="E18" s="8">
         <v>5</v>
       </c>
     </row>
@@ -1350,7 +1353,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="s">
+      <c r="A41" s="6" t="s">
         <v>60</v>
       </c>
       <c r="B41" s="4" t="s">
@@ -1367,7 +1370,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="s">
+      <c r="A42" s="6" t="s">
         <v>61</v>
       </c>
       <c r="B42" s="4" t="s">
@@ -1384,7 +1387,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="s">
+      <c r="A43" s="6" t="s">
         <v>62</v>
       </c>
       <c r="B43" s="4" t="s">
@@ -1401,7 +1404,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="s">
+      <c r="A44" s="6" t="s">
         <v>63</v>
       </c>
       <c r="B44" s="4" t="s">
@@ -1418,7 +1421,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="s">
+      <c r="A45" s="6" t="s">
         <v>64</v>
       </c>
       <c r="B45" s="4" t="s">
@@ -1435,940 +1438,940 @@
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="7"/>
-      <c r="C46" s="7"/>
-      <c r="D46" s="7"/>
-      <c r="E46" s="7"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
     </row>
     <row r="47">
-      <c r="B47" s="7"/>
-      <c r="C47" s="7"/>
-      <c r="D47" s="7"/>
-      <c r="E47" s="7"/>
+      <c r="B47" s="8"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="8"/>
+      <c r="E47" s="8"/>
     </row>
     <row r="48">
-      <c r="B48" s="7"/>
-      <c r="C48" s="7"/>
-      <c r="D48" s="7"/>
-      <c r="E48" s="7"/>
+      <c r="B48" s="8"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
     </row>
     <row r="49">
-      <c r="B49" s="7"/>
-      <c r="C49" s="7"/>
-      <c r="D49" s="7"/>
-      <c r="E49" s="7"/>
+      <c r="B49" s="8"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="8"/>
+      <c r="E49" s="8"/>
     </row>
     <row r="50">
-      <c r="B50" s="7"/>
-      <c r="C50" s="7"/>
-      <c r="D50" s="7"/>
-      <c r="E50" s="7"/>
+      <c r="B50" s="8"/>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8"/>
     </row>
     <row r="51">
-      <c r="B51" s="7"/>
-      <c r="C51" s="7"/>
-      <c r="D51" s="7"/>
-      <c r="E51" s="7"/>
+      <c r="B51" s="8"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="8"/>
+      <c r="E51" s="8"/>
     </row>
     <row r="52">
-      <c r="B52" s="7"/>
-      <c r="C52" s="7"/>
-      <c r="D52" s="7"/>
-      <c r="E52" s="7"/>
+      <c r="B52" s="8"/>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8"/>
     </row>
     <row r="53">
-      <c r="B53" s="7"/>
-      <c r="C53" s="7"/>
-      <c r="D53" s="7"/>
-      <c r="E53" s="7"/>
+      <c r="B53" s="8"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
+      <c r="E53" s="8"/>
     </row>
     <row r="54">
-      <c r="B54" s="7"/>
-      <c r="C54" s="7"/>
-      <c r="D54" s="7"/>
-      <c r="E54" s="7"/>
+      <c r="B54" s="8"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8"/>
     </row>
     <row r="55">
-      <c r="B55" s="7"/>
-      <c r="C55" s="7"/>
-      <c r="D55" s="7"/>
-      <c r="E55" s="7"/>
+      <c r="B55" s="8"/>
+      <c r="C55" s="8"/>
+      <c r="D55" s="8"/>
+      <c r="E55" s="8"/>
     </row>
     <row r="56">
-      <c r="B56" s="7"/>
-      <c r="C56" s="7"/>
-      <c r="D56" s="7"/>
-      <c r="E56" s="7"/>
+      <c r="B56" s="8"/>
+      <c r="C56" s="8"/>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8"/>
     </row>
     <row r="57">
-      <c r="B57" s="7"/>
-      <c r="C57" s="7"/>
-      <c r="D57" s="7"/>
-      <c r="E57" s="7"/>
+      <c r="B57" s="8"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="8"/>
+      <c r="E57" s="8"/>
     </row>
     <row r="58">
-      <c r="B58" s="7"/>
-      <c r="C58" s="7"/>
-      <c r="D58" s="7"/>
-      <c r="E58" s="7"/>
+      <c r="B58" s="8"/>
+      <c r="C58" s="8"/>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8"/>
     </row>
     <row r="59">
-      <c r="B59" s="7"/>
-      <c r="C59" s="7"/>
-      <c r="D59" s="7"/>
-      <c r="E59" s="7"/>
+      <c r="B59" s="8"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="8"/>
+      <c r="E59" s="8"/>
     </row>
     <row r="60">
-      <c r="B60" s="7"/>
-      <c r="C60" s="7"/>
-      <c r="D60" s="7"/>
-      <c r="E60" s="7"/>
+      <c r="B60" s="8"/>
+      <c r="C60" s="8"/>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8"/>
     </row>
     <row r="61">
-      <c r="B61" s="7"/>
-      <c r="C61" s="7"/>
-      <c r="D61" s="7"/>
-      <c r="E61" s="7"/>
+      <c r="B61" s="8"/>
+      <c r="C61" s="8"/>
+      <c r="D61" s="8"/>
+      <c r="E61" s="8"/>
     </row>
     <row r="62">
-      <c r="B62" s="7"/>
-      <c r="C62" s="7"/>
-      <c r="D62" s="7"/>
-      <c r="E62" s="7"/>
+      <c r="B62" s="8"/>
+      <c r="C62" s="8"/>
+      <c r="D62" s="8"/>
+      <c r="E62" s="8"/>
     </row>
     <row r="63">
-      <c r="B63" s="7"/>
-      <c r="C63" s="7"/>
-      <c r="D63" s="7"/>
-      <c r="E63" s="7"/>
+      <c r="B63" s="8"/>
+      <c r="C63" s="8"/>
+      <c r="D63" s="8"/>
+      <c r="E63" s="8"/>
     </row>
     <row r="64">
-      <c r="B64" s="7"/>
-      <c r="C64" s="7"/>
-      <c r="D64" s="7"/>
-      <c r="E64" s="7"/>
+      <c r="B64" s="8"/>
+      <c r="C64" s="8"/>
+      <c r="D64" s="8"/>
+      <c r="E64" s="8"/>
     </row>
     <row r="65">
-      <c r="B65" s="7"/>
-      <c r="C65" s="7"/>
-      <c r="D65" s="7"/>
-      <c r="E65" s="7"/>
+      <c r="B65" s="8"/>
+      <c r="C65" s="8"/>
+      <c r="D65" s="8"/>
+      <c r="E65" s="8"/>
     </row>
     <row r="66">
-      <c r="B66" s="7"/>
-      <c r="C66" s="7"/>
-      <c r="D66" s="7"/>
-      <c r="E66" s="7"/>
+      <c r="B66" s="8"/>
+      <c r="C66" s="8"/>
+      <c r="D66" s="8"/>
+      <c r="E66" s="8"/>
     </row>
     <row r="67">
-      <c r="B67" s="7"/>
-      <c r="C67" s="7"/>
-      <c r="D67" s="7"/>
-      <c r="E67" s="7"/>
+      <c r="B67" s="8"/>
+      <c r="C67" s="8"/>
+      <c r="D67" s="8"/>
+      <c r="E67" s="8"/>
     </row>
     <row r="68">
-      <c r="B68" s="7"/>
-      <c r="C68" s="7"/>
-      <c r="D68" s="7"/>
-      <c r="E68" s="7"/>
+      <c r="B68" s="8"/>
+      <c r="C68" s="8"/>
+      <c r="D68" s="8"/>
+      <c r="E68" s="8"/>
     </row>
     <row r="69">
-      <c r="B69" s="7"/>
-      <c r="C69" s="7"/>
-      <c r="D69" s="7"/>
-      <c r="E69" s="7"/>
+      <c r="B69" s="8"/>
+      <c r="C69" s="8"/>
+      <c r="D69" s="8"/>
+      <c r="E69" s="8"/>
     </row>
     <row r="70">
-      <c r="B70" s="7"/>
-      <c r="C70" s="7"/>
-      <c r="D70" s="7"/>
-      <c r="E70" s="7"/>
+      <c r="B70" s="8"/>
+      <c r="C70" s="8"/>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8"/>
     </row>
     <row r="71">
-      <c r="B71" s="7"/>
-      <c r="C71" s="7"/>
-      <c r="D71" s="7"/>
-      <c r="E71" s="7"/>
+      <c r="B71" s="8"/>
+      <c r="C71" s="8"/>
+      <c r="D71" s="8"/>
+      <c r="E71" s="8"/>
     </row>
     <row r="72">
-      <c r="B72" s="7"/>
-      <c r="C72" s="7"/>
-      <c r="D72" s="7"/>
-      <c r="E72" s="7"/>
+      <c r="B72" s="8"/>
+      <c r="C72" s="8"/>
+      <c r="D72" s="8"/>
+      <c r="E72" s="8"/>
     </row>
     <row r="73">
-      <c r="B73" s="7"/>
-      <c r="C73" s="7"/>
-      <c r="D73" s="7"/>
-      <c r="E73" s="7"/>
+      <c r="B73" s="8"/>
+      <c r="C73" s="8"/>
+      <c r="D73" s="8"/>
+      <c r="E73" s="8"/>
     </row>
     <row r="74">
-      <c r="B74" s="7"/>
-      <c r="C74" s="7"/>
-      <c r="D74" s="7"/>
-      <c r="E74" s="7"/>
+      <c r="B74" s="8"/>
+      <c r="C74" s="8"/>
+      <c r="D74" s="8"/>
+      <c r="E74" s="8"/>
     </row>
     <row r="75">
-      <c r="B75" s="7"/>
-      <c r="C75" s="7"/>
-      <c r="D75" s="7"/>
-      <c r="E75" s="7"/>
+      <c r="B75" s="8"/>
+      <c r="C75" s="8"/>
+      <c r="D75" s="8"/>
+      <c r="E75" s="8"/>
     </row>
     <row r="76">
-      <c r="B76" s="7"/>
-      <c r="C76" s="7"/>
-      <c r="D76" s="7"/>
-      <c r="E76" s="7"/>
+      <c r="B76" s="8"/>
+      <c r="C76" s="8"/>
+      <c r="D76" s="8"/>
+      <c r="E76" s="8"/>
     </row>
     <row r="77">
-      <c r="B77" s="7"/>
-      <c r="C77" s="7"/>
-      <c r="D77" s="7"/>
-      <c r="E77" s="7"/>
+      <c r="B77" s="8"/>
+      <c r="C77" s="8"/>
+      <c r="D77" s="8"/>
+      <c r="E77" s="8"/>
     </row>
     <row r="78">
-      <c r="B78" s="7"/>
-      <c r="C78" s="7"/>
-      <c r="D78" s="7"/>
-      <c r="E78" s="7"/>
+      <c r="B78" s="8"/>
+      <c r="C78" s="8"/>
+      <c r="D78" s="8"/>
+      <c r="E78" s="8"/>
     </row>
     <row r="79">
-      <c r="B79" s="7"/>
-      <c r="C79" s="7"/>
-      <c r="D79" s="7"/>
-      <c r="E79" s="7"/>
+      <c r="B79" s="8"/>
+      <c r="C79" s="8"/>
+      <c r="D79" s="8"/>
+      <c r="E79" s="8"/>
     </row>
     <row r="80">
-      <c r="B80" s="7"/>
-      <c r="C80" s="7"/>
-      <c r="D80" s="7"/>
-      <c r="E80" s="7"/>
+      <c r="B80" s="8"/>
+      <c r="C80" s="8"/>
+      <c r="D80" s="8"/>
+      <c r="E80" s="8"/>
     </row>
     <row r="81">
-      <c r="B81" s="7"/>
-      <c r="C81" s="7"/>
-      <c r="D81" s="7"/>
-      <c r="E81" s="7"/>
+      <c r="B81" s="8"/>
+      <c r="C81" s="8"/>
+      <c r="D81" s="8"/>
+      <c r="E81" s="8"/>
     </row>
     <row r="82">
-      <c r="B82" s="7"/>
-      <c r="C82" s="7"/>
-      <c r="D82" s="7"/>
-      <c r="E82" s="7"/>
+      <c r="B82" s="8"/>
+      <c r="C82" s="8"/>
+      <c r="D82" s="8"/>
+      <c r="E82" s="8"/>
     </row>
     <row r="83">
-      <c r="B83" s="7"/>
-      <c r="C83" s="7"/>
-      <c r="D83" s="7"/>
-      <c r="E83" s="7"/>
+      <c r="B83" s="8"/>
+      <c r="C83" s="8"/>
+      <c r="D83" s="8"/>
+      <c r="E83" s="8"/>
     </row>
     <row r="84">
-      <c r="B84" s="7"/>
-      <c r="C84" s="7"/>
-      <c r="D84" s="7"/>
-      <c r="E84" s="7"/>
+      <c r="B84" s="8"/>
+      <c r="C84" s="8"/>
+      <c r="D84" s="8"/>
+      <c r="E84" s="8"/>
     </row>
     <row r="85">
-      <c r="B85" s="7"/>
-      <c r="C85" s="7"/>
-      <c r="D85" s="7"/>
-      <c r="E85" s="7"/>
+      <c r="B85" s="8"/>
+      <c r="C85" s="8"/>
+      <c r="D85" s="8"/>
+      <c r="E85" s="8"/>
     </row>
     <row r="86">
-      <c r="B86" s="7"/>
-      <c r="C86" s="7"/>
-      <c r="D86" s="7"/>
-      <c r="E86" s="7"/>
+      <c r="B86" s="8"/>
+      <c r="C86" s="8"/>
+      <c r="D86" s="8"/>
+      <c r="E86" s="8"/>
     </row>
     <row r="87">
-      <c r="B87" s="7"/>
-      <c r="C87" s="7"/>
-      <c r="D87" s="7"/>
-      <c r="E87" s="7"/>
+      <c r="B87" s="8"/>
+      <c r="C87" s="8"/>
+      <c r="D87" s="8"/>
+      <c r="E87" s="8"/>
     </row>
     <row r="88">
-      <c r="B88" s="7"/>
-      <c r="C88" s="7"/>
-      <c r="D88" s="7"/>
-      <c r="E88" s="7"/>
+      <c r="B88" s="8"/>
+      <c r="C88" s="8"/>
+      <c r="D88" s="8"/>
+      <c r="E88" s="8"/>
     </row>
     <row r="89">
-      <c r="B89" s="7"/>
-      <c r="C89" s="7"/>
-      <c r="D89" s="7"/>
-      <c r="E89" s="7"/>
+      <c r="B89" s="8"/>
+      <c r="C89" s="8"/>
+      <c r="D89" s="8"/>
+      <c r="E89" s="8"/>
     </row>
     <row r="90">
-      <c r="B90" s="7"/>
-      <c r="C90" s="7"/>
-      <c r="D90" s="7"/>
-      <c r="E90" s="7"/>
+      <c r="B90" s="8"/>
+      <c r="C90" s="8"/>
+      <c r="D90" s="8"/>
+      <c r="E90" s="8"/>
     </row>
     <row r="91">
-      <c r="B91" s="7"/>
-      <c r="C91" s="7"/>
-      <c r="D91" s="7"/>
-      <c r="E91" s="7"/>
+      <c r="B91" s="8"/>
+      <c r="C91" s="8"/>
+      <c r="D91" s="8"/>
+      <c r="E91" s="8"/>
     </row>
     <row r="92">
-      <c r="B92" s="7"/>
-      <c r="C92" s="7"/>
-      <c r="D92" s="7"/>
-      <c r="E92" s="7"/>
+      <c r="B92" s="8"/>
+      <c r="C92" s="8"/>
+      <c r="D92" s="8"/>
+      <c r="E92" s="8"/>
     </row>
     <row r="93">
-      <c r="B93" s="7"/>
-      <c r="C93" s="7"/>
-      <c r="D93" s="7"/>
-      <c r="E93" s="7"/>
+      <c r="B93" s="8"/>
+      <c r="C93" s="8"/>
+      <c r="D93" s="8"/>
+      <c r="E93" s="8"/>
     </row>
     <row r="94">
-      <c r="B94" s="7"/>
-      <c r="C94" s="7"/>
-      <c r="D94" s="7"/>
-      <c r="E94" s="7"/>
+      <c r="B94" s="8"/>
+      <c r="C94" s="8"/>
+      <c r="D94" s="8"/>
+      <c r="E94" s="8"/>
     </row>
     <row r="95">
-      <c r="B95" s="7"/>
-      <c r="C95" s="7"/>
-      <c r="D95" s="7"/>
-      <c r="E95" s="7"/>
+      <c r="B95" s="8"/>
+      <c r="C95" s="8"/>
+      <c r="D95" s="8"/>
+      <c r="E95" s="8"/>
     </row>
     <row r="96">
-      <c r="B96" s="7"/>
-      <c r="C96" s="7"/>
-      <c r="D96" s="7"/>
-      <c r="E96" s="7"/>
+      <c r="B96" s="8"/>
+      <c r="C96" s="8"/>
+      <c r="D96" s="8"/>
+      <c r="E96" s="8"/>
     </row>
     <row r="97">
-      <c r="B97" s="7"/>
-      <c r="C97" s="7"/>
-      <c r="D97" s="7"/>
-      <c r="E97" s="7"/>
+      <c r="B97" s="8"/>
+      <c r="C97" s="8"/>
+      <c r="D97" s="8"/>
+      <c r="E97" s="8"/>
     </row>
     <row r="98">
-      <c r="B98" s="7"/>
-      <c r="C98" s="7"/>
-      <c r="D98" s="7"/>
-      <c r="E98" s="7"/>
+      <c r="B98" s="8"/>
+      <c r="C98" s="8"/>
+      <c r="D98" s="8"/>
+      <c r="E98" s="8"/>
     </row>
     <row r="99">
-      <c r="B99" s="7"/>
-      <c r="C99" s="7"/>
-      <c r="D99" s="7"/>
-      <c r="E99" s="7"/>
+      <c r="B99" s="8"/>
+      <c r="C99" s="8"/>
+      <c r="D99" s="8"/>
+      <c r="E99" s="8"/>
     </row>
     <row r="100">
-      <c r="B100" s="7"/>
-      <c r="C100" s="7"/>
-      <c r="D100" s="7"/>
-      <c r="E100" s="7"/>
+      <c r="B100" s="8"/>
+      <c r="C100" s="8"/>
+      <c r="D100" s="8"/>
+      <c r="E100" s="8"/>
     </row>
     <row r="101">
-      <c r="B101" s="7"/>
-      <c r="C101" s="7"/>
-      <c r="D101" s="7"/>
-      <c r="E101" s="7"/>
+      <c r="B101" s="8"/>
+      <c r="C101" s="8"/>
+      <c r="D101" s="8"/>
+      <c r="E101" s="8"/>
     </row>
     <row r="102">
-      <c r="B102" s="7"/>
-      <c r="C102" s="7"/>
-      <c r="D102" s="7"/>
-      <c r="E102" s="7"/>
+      <c r="B102" s="8"/>
+      <c r="C102" s="8"/>
+      <c r="D102" s="8"/>
+      <c r="E102" s="8"/>
     </row>
     <row r="103">
-      <c r="B103" s="7"/>
-      <c r="C103" s="7"/>
-      <c r="D103" s="7"/>
-      <c r="E103" s="7"/>
+      <c r="B103" s="8"/>
+      <c r="C103" s="8"/>
+      <c r="D103" s="8"/>
+      <c r="E103" s="8"/>
     </row>
     <row r="104">
-      <c r="B104" s="7"/>
-      <c r="C104" s="7"/>
-      <c r="D104" s="7"/>
-      <c r="E104" s="7"/>
+      <c r="B104" s="8"/>
+      <c r="C104" s="8"/>
+      <c r="D104" s="8"/>
+      <c r="E104" s="8"/>
     </row>
     <row r="105">
-      <c r="B105" s="7"/>
-      <c r="C105" s="7"/>
-      <c r="D105" s="7"/>
-      <c r="E105" s="7"/>
+      <c r="B105" s="8"/>
+      <c r="C105" s="8"/>
+      <c r="D105" s="8"/>
+      <c r="E105" s="8"/>
     </row>
     <row r="106">
-      <c r="B106" s="7"/>
-      <c r="C106" s="7"/>
-      <c r="D106" s="7"/>
-      <c r="E106" s="7"/>
+      <c r="B106" s="8"/>
+      <c r="C106" s="8"/>
+      <c r="D106" s="8"/>
+      <c r="E106" s="8"/>
     </row>
     <row r="107">
-      <c r="B107" s="7"/>
-      <c r="C107" s="7"/>
-      <c r="D107" s="7"/>
-      <c r="E107" s="7"/>
+      <c r="B107" s="8"/>
+      <c r="C107" s="8"/>
+      <c r="D107" s="8"/>
+      <c r="E107" s="8"/>
     </row>
     <row r="108">
-      <c r="B108" s="7"/>
-      <c r="C108" s="7"/>
-      <c r="D108" s="7"/>
-      <c r="E108" s="7"/>
+      <c r="B108" s="8"/>
+      <c r="C108" s="8"/>
+      <c r="D108" s="8"/>
+      <c r="E108" s="8"/>
     </row>
     <row r="109">
-      <c r="B109" s="7"/>
-      <c r="C109" s="7"/>
-      <c r="D109" s="7"/>
-      <c r="E109" s="7"/>
+      <c r="B109" s="8"/>
+      <c r="C109" s="8"/>
+      <c r="D109" s="8"/>
+      <c r="E109" s="8"/>
     </row>
     <row r="110">
-      <c r="B110" s="7"/>
-      <c r="C110" s="7"/>
-      <c r="D110" s="7"/>
-      <c r="E110" s="7"/>
+      <c r="B110" s="8"/>
+      <c r="C110" s="8"/>
+      <c r="D110" s="8"/>
+      <c r="E110" s="8"/>
     </row>
     <row r="111">
-      <c r="B111" s="7"/>
-      <c r="C111" s="7"/>
-      <c r="D111" s="7"/>
-      <c r="E111" s="7"/>
+      <c r="B111" s="8"/>
+      <c r="C111" s="8"/>
+      <c r="D111" s="8"/>
+      <c r="E111" s="8"/>
     </row>
     <row r="112">
-      <c r="B112" s="7"/>
-      <c r="C112" s="7"/>
-      <c r="D112" s="7"/>
-      <c r="E112" s="7"/>
+      <c r="B112" s="8"/>
+      <c r="C112" s="8"/>
+      <c r="D112" s="8"/>
+      <c r="E112" s="8"/>
     </row>
     <row r="113">
-      <c r="B113" s="7"/>
-      <c r="C113" s="7"/>
-      <c r="D113" s="7"/>
-      <c r="E113" s="7"/>
+      <c r="B113" s="8"/>
+      <c r="C113" s="8"/>
+      <c r="D113" s="8"/>
+      <c r="E113" s="8"/>
     </row>
     <row r="114">
-      <c r="B114" s="7"/>
-      <c r="C114" s="7"/>
-      <c r="D114" s="7"/>
-      <c r="E114" s="7"/>
+      <c r="B114" s="8"/>
+      <c r="C114" s="8"/>
+      <c r="D114" s="8"/>
+      <c r="E114" s="8"/>
     </row>
     <row r="115">
-      <c r="B115" s="7"/>
-      <c r="C115" s="7"/>
-      <c r="D115" s="7"/>
-      <c r="E115" s="7"/>
+      <c r="B115" s="8"/>
+      <c r="C115" s="8"/>
+      <c r="D115" s="8"/>
+      <c r="E115" s="8"/>
     </row>
     <row r="116">
-      <c r="B116" s="7"/>
-      <c r="C116" s="7"/>
-      <c r="D116" s="7"/>
-      <c r="E116" s="7"/>
+      <c r="B116" s="8"/>
+      <c r="C116" s="8"/>
+      <c r="D116" s="8"/>
+      <c r="E116" s="8"/>
     </row>
     <row r="117">
-      <c r="B117" s="7"/>
-      <c r="C117" s="7"/>
-      <c r="D117" s="7"/>
-      <c r="E117" s="7"/>
+      <c r="B117" s="8"/>
+      <c r="C117" s="8"/>
+      <c r="D117" s="8"/>
+      <c r="E117" s="8"/>
     </row>
     <row r="118">
-      <c r="B118" s="7"/>
-      <c r="C118" s="7"/>
-      <c r="D118" s="7"/>
-      <c r="E118" s="7"/>
+      <c r="B118" s="8"/>
+      <c r="C118" s="8"/>
+      <c r="D118" s="8"/>
+      <c r="E118" s="8"/>
     </row>
     <row r="119">
-      <c r="B119" s="7"/>
-      <c r="C119" s="7"/>
-      <c r="D119" s="7"/>
-      <c r="E119" s="7"/>
+      <c r="B119" s="8"/>
+      <c r="C119" s="8"/>
+      <c r="D119" s="8"/>
+      <c r="E119" s="8"/>
     </row>
     <row r="120">
-      <c r="B120" s="7"/>
-      <c r="C120" s="7"/>
-      <c r="D120" s="7"/>
-      <c r="E120" s="7"/>
+      <c r="B120" s="8"/>
+      <c r="C120" s="8"/>
+      <c r="D120" s="8"/>
+      <c r="E120" s="8"/>
     </row>
     <row r="121">
-      <c r="B121" s="7"/>
-      <c r="C121" s="7"/>
-      <c r="D121" s="7"/>
-      <c r="E121" s="7"/>
+      <c r="B121" s="8"/>
+      <c r="C121" s="8"/>
+      <c r="D121" s="8"/>
+      <c r="E121" s="8"/>
     </row>
     <row r="122">
-      <c r="B122" s="7"/>
-      <c r="C122" s="7"/>
-      <c r="D122" s="7"/>
-      <c r="E122" s="7"/>
+      <c r="B122" s="8"/>
+      <c r="C122" s="8"/>
+      <c r="D122" s="8"/>
+      <c r="E122" s="8"/>
     </row>
     <row r="123">
-      <c r="B123" s="7"/>
-      <c r="C123" s="7"/>
-      <c r="D123" s="7"/>
-      <c r="E123" s="7"/>
+      <c r="B123" s="8"/>
+      <c r="C123" s="8"/>
+      <c r="D123" s="8"/>
+      <c r="E123" s="8"/>
     </row>
     <row r="124">
-      <c r="B124" s="7"/>
-      <c r="C124" s="7"/>
-      <c r="D124" s="7"/>
-      <c r="E124" s="7"/>
+      <c r="B124" s="8"/>
+      <c r="C124" s="8"/>
+      <c r="D124" s="8"/>
+      <c r="E124" s="8"/>
     </row>
     <row r="125">
-      <c r="B125" s="7"/>
-      <c r="C125" s="7"/>
-      <c r="D125" s="7"/>
-      <c r="E125" s="7"/>
+      <c r="B125" s="8"/>
+      <c r="C125" s="8"/>
+      <c r="D125" s="8"/>
+      <c r="E125" s="8"/>
     </row>
     <row r="126">
-      <c r="B126" s="7"/>
-      <c r="C126" s="7"/>
-      <c r="D126" s="7"/>
-      <c r="E126" s="7"/>
+      <c r="B126" s="8"/>
+      <c r="C126" s="8"/>
+      <c r="D126" s="8"/>
+      <c r="E126" s="8"/>
     </row>
     <row r="127">
-      <c r="B127" s="7"/>
-      <c r="C127" s="7"/>
-      <c r="D127" s="7"/>
-      <c r="E127" s="7"/>
+      <c r="B127" s="8"/>
+      <c r="C127" s="8"/>
+      <c r="D127" s="8"/>
+      <c r="E127" s="8"/>
     </row>
     <row r="128">
-      <c r="B128" s="7"/>
-      <c r="C128" s="7"/>
-      <c r="D128" s="7"/>
-      <c r="E128" s="7"/>
+      <c r="B128" s="8"/>
+      <c r="C128" s="8"/>
+      <c r="D128" s="8"/>
+      <c r="E128" s="8"/>
     </row>
     <row r="129">
-      <c r="B129" s="7"/>
-      <c r="C129" s="7"/>
-      <c r="D129" s="7"/>
-      <c r="E129" s="7"/>
+      <c r="B129" s="8"/>
+      <c r="C129" s="8"/>
+      <c r="D129" s="8"/>
+      <c r="E129" s="8"/>
     </row>
     <row r="130">
-      <c r="B130" s="7"/>
-      <c r="C130" s="7"/>
-      <c r="D130" s="7"/>
-      <c r="E130" s="7"/>
+      <c r="B130" s="8"/>
+      <c r="C130" s="8"/>
+      <c r="D130" s="8"/>
+      <c r="E130" s="8"/>
     </row>
     <row r="131">
-      <c r="B131" s="7"/>
-      <c r="C131" s="7"/>
-      <c r="D131" s="7"/>
-      <c r="E131" s="7"/>
+      <c r="B131" s="8"/>
+      <c r="C131" s="8"/>
+      <c r="D131" s="8"/>
+      <c r="E131" s="8"/>
     </row>
     <row r="132">
-      <c r="B132" s="7"/>
-      <c r="C132" s="7"/>
-      <c r="D132" s="7"/>
-      <c r="E132" s="7"/>
+      <c r="B132" s="8"/>
+      <c r="C132" s="8"/>
+      <c r="D132" s="8"/>
+      <c r="E132" s="8"/>
     </row>
     <row r="133">
-      <c r="B133" s="7"/>
-      <c r="C133" s="7"/>
-      <c r="D133" s="7"/>
-      <c r="E133" s="7"/>
+      <c r="B133" s="8"/>
+      <c r="C133" s="8"/>
+      <c r="D133" s="8"/>
+      <c r="E133" s="8"/>
     </row>
     <row r="134">
-      <c r="B134" s="7"/>
-      <c r="C134" s="7"/>
-      <c r="D134" s="7"/>
-      <c r="E134" s="7"/>
+      <c r="B134" s="8"/>
+      <c r="C134" s="8"/>
+      <c r="D134" s="8"/>
+      <c r="E134" s="8"/>
     </row>
     <row r="135">
-      <c r="B135" s="7"/>
-      <c r="C135" s="7"/>
-      <c r="D135" s="7"/>
-      <c r="E135" s="7"/>
+      <c r="B135" s="8"/>
+      <c r="C135" s="8"/>
+      <c r="D135" s="8"/>
+      <c r="E135" s="8"/>
     </row>
     <row r="136">
-      <c r="B136" s="7"/>
-      <c r="C136" s="7"/>
-      <c r="D136" s="7"/>
-      <c r="E136" s="7"/>
+      <c r="B136" s="8"/>
+      <c r="C136" s="8"/>
+      <c r="D136" s="8"/>
+      <c r="E136" s="8"/>
     </row>
     <row r="137">
-      <c r="B137" s="7"/>
-      <c r="C137" s="7"/>
-      <c r="D137" s="7"/>
-      <c r="E137" s="7"/>
+      <c r="B137" s="8"/>
+      <c r="C137" s="8"/>
+      <c r="D137" s="8"/>
+      <c r="E137" s="8"/>
     </row>
     <row r="138">
-      <c r="B138" s="7"/>
-      <c r="C138" s="7"/>
-      <c r="D138" s="7"/>
-      <c r="E138" s="7"/>
+      <c r="B138" s="8"/>
+      <c r="C138" s="8"/>
+      <c r="D138" s="8"/>
+      <c r="E138" s="8"/>
     </row>
     <row r="139">
-      <c r="B139" s="7"/>
-      <c r="C139" s="7"/>
-      <c r="D139" s="7"/>
-      <c r="E139" s="7"/>
+      <c r="B139" s="8"/>
+      <c r="C139" s="8"/>
+      <c r="D139" s="8"/>
+      <c r="E139" s="8"/>
     </row>
     <row r="140">
-      <c r="B140" s="7"/>
-      <c r="C140" s="7"/>
-      <c r="D140" s="7"/>
-      <c r="E140" s="7"/>
+      <c r="B140" s="8"/>
+      <c r="C140" s="8"/>
+      <c r="D140" s="8"/>
+      <c r="E140" s="8"/>
     </row>
     <row r="141">
-      <c r="B141" s="7"/>
-      <c r="C141" s="7"/>
-      <c r="D141" s="7"/>
-      <c r="E141" s="7"/>
+      <c r="B141" s="8"/>
+      <c r="C141" s="8"/>
+      <c r="D141" s="8"/>
+      <c r="E141" s="8"/>
     </row>
     <row r="142">
-      <c r="B142" s="7"/>
-      <c r="C142" s="7"/>
-      <c r="D142" s="7"/>
-      <c r="E142" s="7"/>
+      <c r="B142" s="8"/>
+      <c r="C142" s="8"/>
+      <c r="D142" s="8"/>
+      <c r="E142" s="8"/>
     </row>
     <row r="143">
-      <c r="B143" s="7"/>
-      <c r="C143" s="7"/>
-      <c r="D143" s="7"/>
-      <c r="E143" s="7"/>
+      <c r="B143" s="8"/>
+      <c r="C143" s="8"/>
+      <c r="D143" s="8"/>
+      <c r="E143" s="8"/>
     </row>
     <row r="144">
-      <c r="B144" s="7"/>
-      <c r="C144" s="7"/>
-      <c r="D144" s="7"/>
-      <c r="E144" s="7"/>
+      <c r="B144" s="8"/>
+      <c r="C144" s="8"/>
+      <c r="D144" s="8"/>
+      <c r="E144" s="8"/>
     </row>
     <row r="145">
-      <c r="B145" s="7"/>
-      <c r="C145" s="7"/>
-      <c r="D145" s="7"/>
-      <c r="E145" s="7"/>
+      <c r="B145" s="8"/>
+      <c r="C145" s="8"/>
+      <c r="D145" s="8"/>
+      <c r="E145" s="8"/>
     </row>
     <row r="146">
-      <c r="B146" s="7"/>
-      <c r="C146" s="7"/>
-      <c r="D146" s="7"/>
-      <c r="E146" s="7"/>
+      <c r="B146" s="8"/>
+      <c r="C146" s="8"/>
+      <c r="D146" s="8"/>
+      <c r="E146" s="8"/>
     </row>
     <row r="147">
-      <c r="B147" s="7"/>
-      <c r="C147" s="7"/>
-      <c r="D147" s="7"/>
-      <c r="E147" s="7"/>
+      <c r="B147" s="8"/>
+      <c r="C147" s="8"/>
+      <c r="D147" s="8"/>
+      <c r="E147" s="8"/>
     </row>
     <row r="148">
-      <c r="B148" s="7"/>
-      <c r="C148" s="7"/>
-      <c r="D148" s="7"/>
-      <c r="E148" s="7"/>
+      <c r="B148" s="8"/>
+      <c r="C148" s="8"/>
+      <c r="D148" s="8"/>
+      <c r="E148" s="8"/>
     </row>
     <row r="149">
-      <c r="B149" s="7"/>
-      <c r="C149" s="7"/>
-      <c r="D149" s="7"/>
-      <c r="E149" s="7"/>
+      <c r="B149" s="8"/>
+      <c r="C149" s="8"/>
+      <c r="D149" s="8"/>
+      <c r="E149" s="8"/>
     </row>
     <row r="150">
-      <c r="B150" s="7"/>
-      <c r="C150" s="7"/>
-      <c r="D150" s="7"/>
-      <c r="E150" s="7"/>
+      <c r="B150" s="8"/>
+      <c r="C150" s="8"/>
+      <c r="D150" s="8"/>
+      <c r="E150" s="8"/>
     </row>
     <row r="151">
-      <c r="B151" s="7"/>
-      <c r="C151" s="7"/>
-      <c r="D151" s="7"/>
-      <c r="E151" s="7"/>
+      <c r="B151" s="8"/>
+      <c r="C151" s="8"/>
+      <c r="D151" s="8"/>
+      <c r="E151" s="8"/>
     </row>
     <row r="152">
-      <c r="B152" s="7"/>
-      <c r="C152" s="7"/>
-      <c r="D152" s="7"/>
-      <c r="E152" s="7"/>
+      <c r="B152" s="8"/>
+      <c r="C152" s="8"/>
+      <c r="D152" s="8"/>
+      <c r="E152" s="8"/>
     </row>
     <row r="153">
-      <c r="B153" s="7"/>
-      <c r="C153" s="7"/>
-      <c r="D153" s="7"/>
-      <c r="E153" s="7"/>
+      <c r="B153" s="8"/>
+      <c r="C153" s="8"/>
+      <c r="D153" s="8"/>
+      <c r="E153" s="8"/>
     </row>
     <row r="154">
-      <c r="B154" s="7"/>
-      <c r="C154" s="7"/>
-      <c r="D154" s="7"/>
-      <c r="E154" s="7"/>
+      <c r="B154" s="8"/>
+      <c r="C154" s="8"/>
+      <c r="D154" s="8"/>
+      <c r="E154" s="8"/>
     </row>
     <row r="155">
-      <c r="B155" s="7"/>
-      <c r="C155" s="7"/>
-      <c r="D155" s="7"/>
-      <c r="E155" s="7"/>
+      <c r="B155" s="8"/>
+      <c r="C155" s="8"/>
+      <c r="D155" s="8"/>
+      <c r="E155" s="8"/>
     </row>
     <row r="156">
-      <c r="B156" s="7"/>
-      <c r="C156" s="7"/>
-      <c r="D156" s="7"/>
-      <c r="E156" s="7"/>
+      <c r="B156" s="8"/>
+      <c r="C156" s="8"/>
+      <c r="D156" s="8"/>
+      <c r="E156" s="8"/>
     </row>
     <row r="157">
-      <c r="B157" s="7"/>
-      <c r="C157" s="7"/>
-      <c r="D157" s="7"/>
-      <c r="E157" s="7"/>
+      <c r="B157" s="8"/>
+      <c r="C157" s="8"/>
+      <c r="D157" s="8"/>
+      <c r="E157" s="8"/>
     </row>
     <row r="158">
-      <c r="B158" s="7"/>
-      <c r="C158" s="7"/>
-      <c r="D158" s="7"/>
-      <c r="E158" s="7"/>
+      <c r="B158" s="8"/>
+      <c r="C158" s="8"/>
+      <c r="D158" s="8"/>
+      <c r="E158" s="8"/>
     </row>
     <row r="159">
-      <c r="B159" s="7"/>
-      <c r="C159" s="7"/>
-      <c r="D159" s="7"/>
-      <c r="E159" s="7"/>
+      <c r="B159" s="8"/>
+      <c r="C159" s="8"/>
+      <c r="D159" s="8"/>
+      <c r="E159" s="8"/>
     </row>
     <row r="160">
-      <c r="B160" s="7"/>
-      <c r="C160" s="7"/>
-      <c r="D160" s="7"/>
-      <c r="E160" s="7"/>
+      <c r="B160" s="8"/>
+      <c r="C160" s="8"/>
+      <c r="D160" s="8"/>
+      <c r="E160" s="8"/>
     </row>
     <row r="161">
-      <c r="B161" s="7"/>
-      <c r="C161" s="7"/>
-      <c r="D161" s="7"/>
-      <c r="E161" s="7"/>
+      <c r="B161" s="8"/>
+      <c r="C161" s="8"/>
+      <c r="D161" s="8"/>
+      <c r="E161" s="8"/>
     </row>
     <row r="162">
-      <c r="B162" s="7"/>
-      <c r="C162" s="7"/>
-      <c r="D162" s="7"/>
-      <c r="E162" s="7"/>
+      <c r="B162" s="8"/>
+      <c r="C162" s="8"/>
+      <c r="D162" s="8"/>
+      <c r="E162" s="8"/>
     </row>
     <row r="163">
-      <c r="B163" s="7"/>
-      <c r="C163" s="7"/>
-      <c r="D163" s="7"/>
-      <c r="E163" s="7"/>
+      <c r="B163" s="8"/>
+      <c r="C163" s="8"/>
+      <c r="D163" s="8"/>
+      <c r="E163" s="8"/>
     </row>
     <row r="164">
-      <c r="B164" s="7"/>
-      <c r="C164" s="7"/>
-      <c r="D164" s="7"/>
-      <c r="E164" s="7"/>
+      <c r="B164" s="8"/>
+      <c r="C164" s="8"/>
+      <c r="D164" s="8"/>
+      <c r="E164" s="8"/>
     </row>
     <row r="165">
-      <c r="B165" s="7"/>
-      <c r="C165" s="7"/>
-      <c r="D165" s="7"/>
-      <c r="E165" s="7"/>
+      <c r="B165" s="8"/>
+      <c r="C165" s="8"/>
+      <c r="D165" s="8"/>
+      <c r="E165" s="8"/>
     </row>
     <row r="166">
-      <c r="B166" s="7"/>
-      <c r="C166" s="7"/>
-      <c r="D166" s="7"/>
-      <c r="E166" s="7"/>
+      <c r="B166" s="8"/>
+      <c r="C166" s="8"/>
+      <c r="D166" s="8"/>
+      <c r="E166" s="8"/>
     </row>
     <row r="167">
-      <c r="B167" s="7"/>
-      <c r="C167" s="7"/>
-      <c r="D167" s="7"/>
-      <c r="E167" s="7"/>
+      <c r="B167" s="8"/>
+      <c r="C167" s="8"/>
+      <c r="D167" s="8"/>
+      <c r="E167" s="8"/>
     </row>
     <row r="168">
-      <c r="B168" s="7"/>
-      <c r="C168" s="7"/>
-      <c r="D168" s="7"/>
-      <c r="E168" s="7"/>
+      <c r="B168" s="8"/>
+      <c r="C168" s="8"/>
+      <c r="D168" s="8"/>
+      <c r="E168" s="8"/>
     </row>
     <row r="169">
-      <c r="B169" s="7"/>
-      <c r="C169" s="7"/>
-      <c r="D169" s="7"/>
-      <c r="E169" s="7"/>
+      <c r="B169" s="8"/>
+      <c r="C169" s="8"/>
+      <c r="D169" s="8"/>
+      <c r="E169" s="8"/>
     </row>
     <row r="170">
-      <c r="B170" s="7"/>
-      <c r="C170" s="7"/>
-      <c r="D170" s="7"/>
-      <c r="E170" s="7"/>
+      <c r="B170" s="8"/>
+      <c r="C170" s="8"/>
+      <c r="D170" s="8"/>
+      <c r="E170" s="8"/>
     </row>
     <row r="171">
-      <c r="B171" s="7"/>
-      <c r="C171" s="7"/>
-      <c r="D171" s="7"/>
-      <c r="E171" s="7"/>
+      <c r="B171" s="8"/>
+      <c r="C171" s="8"/>
+      <c r="D171" s="8"/>
+      <c r="E171" s="8"/>
     </row>
     <row r="172">
-      <c r="B172" s="7"/>
-      <c r="C172" s="7"/>
-      <c r="D172" s="7"/>
-      <c r="E172" s="7"/>
+      <c r="B172" s="8"/>
+      <c r="C172" s="8"/>
+      <c r="D172" s="8"/>
+      <c r="E172" s="8"/>
     </row>
     <row r="173">
-      <c r="B173" s="7"/>
-      <c r="C173" s="7"/>
-      <c r="D173" s="7"/>
-      <c r="E173" s="7"/>
+      <c r="B173" s="8"/>
+      <c r="C173" s="8"/>
+      <c r="D173" s="8"/>
+      <c r="E173" s="8"/>
     </row>
     <row r="174">
-      <c r="B174" s="7"/>
-      <c r="C174" s="7"/>
-      <c r="D174" s="7"/>
-      <c r="E174" s="7"/>
+      <c r="B174" s="8"/>
+      <c r="C174" s="8"/>
+      <c r="D174" s="8"/>
+      <c r="E174" s="8"/>
     </row>
     <row r="175">
-      <c r="B175" s="7"/>
-      <c r="C175" s="7"/>
-      <c r="D175" s="7"/>
-      <c r="E175" s="7"/>
+      <c r="B175" s="8"/>
+      <c r="C175" s="8"/>
+      <c r="D175" s="8"/>
+      <c r="E175" s="8"/>
     </row>
     <row r="176">
-      <c r="B176" s="7"/>
-      <c r="C176" s="7"/>
-      <c r="D176" s="7"/>
-      <c r="E176" s="7"/>
+      <c r="B176" s="8"/>
+      <c r="C176" s="8"/>
+      <c r="D176" s="8"/>
+      <c r="E176" s="8"/>
     </row>
     <row r="177">
-      <c r="B177" s="7"/>
-      <c r="C177" s="7"/>
-      <c r="D177" s="7"/>
-      <c r="E177" s="7"/>
+      <c r="B177" s="8"/>
+      <c r="C177" s="8"/>
+      <c r="D177" s="8"/>
+      <c r="E177" s="8"/>
     </row>
     <row r="178">
-      <c r="B178" s="7"/>
-      <c r="C178" s="7"/>
-      <c r="D178" s="7"/>
-      <c r="E178" s="7"/>
+      <c r="B178" s="8"/>
+      <c r="C178" s="8"/>
+      <c r="D178" s="8"/>
+      <c r="E178" s="8"/>
     </row>
     <row r="179">
-      <c r="B179" s="7"/>
-      <c r="C179" s="7"/>
-      <c r="D179" s="7"/>
-      <c r="E179" s="7"/>
+      <c r="B179" s="8"/>
+      <c r="C179" s="8"/>
+      <c r="D179" s="8"/>
+      <c r="E179" s="8"/>
     </row>
     <row r="180">
-      <c r="B180" s="7"/>
-      <c r="C180" s="7"/>
-      <c r="D180" s="7"/>
-      <c r="E180" s="7"/>
+      <c r="B180" s="8"/>
+      <c r="C180" s="8"/>
+      <c r="D180" s="8"/>
+      <c r="E180" s="8"/>
     </row>
     <row r="181">
-      <c r="B181" s="7"/>
-      <c r="C181" s="7"/>
-      <c r="D181" s="7"/>
-      <c r="E181" s="7"/>
+      <c r="B181" s="8"/>
+      <c r="C181" s="8"/>
+      <c r="D181" s="8"/>
+      <c r="E181" s="8"/>
     </row>
     <row r="182">
-      <c r="B182" s="7"/>
-      <c r="C182" s="7"/>
-      <c r="D182" s="7"/>
-      <c r="E182" s="7"/>
+      <c r="B182" s="8"/>
+      <c r="C182" s="8"/>
+      <c r="D182" s="8"/>
+      <c r="E182" s="8"/>
     </row>
     <row r="183">
-      <c r="B183" s="7"/>
-      <c r="C183" s="7"/>
-      <c r="D183" s="7"/>
-      <c r="E183" s="7"/>
+      <c r="B183" s="8"/>
+      <c r="C183" s="8"/>
+      <c r="D183" s="8"/>
+      <c r="E183" s="8"/>
     </row>
     <row r="184">
-      <c r="B184" s="7"/>
-      <c r="C184" s="7"/>
-      <c r="D184" s="7"/>
-      <c r="E184" s="7"/>
+      <c r="B184" s="8"/>
+      <c r="C184" s="8"/>
+      <c r="D184" s="8"/>
+      <c r="E184" s="8"/>
     </row>
     <row r="185">
-      <c r="B185" s="7"/>
-      <c r="C185" s="7"/>
-      <c r="D185" s="7"/>
-      <c r="E185" s="7"/>
+      <c r="B185" s="8"/>
+      <c r="C185" s="8"/>
+      <c r="D185" s="8"/>
+      <c r="E185" s="8"/>
     </row>
     <row r="186">
-      <c r="B186" s="7"/>
-      <c r="C186" s="7"/>
-      <c r="D186" s="7"/>
-      <c r="E186" s="7"/>
+      <c r="B186" s="8"/>
+      <c r="C186" s="8"/>
+      <c r="D186" s="8"/>
+      <c r="E186" s="8"/>
     </row>
     <row r="187">
-      <c r="B187" s="7"/>
-      <c r="C187" s="7"/>
-      <c r="D187" s="7"/>
-      <c r="E187" s="7"/>
+      <c r="B187" s="8"/>
+      <c r="C187" s="8"/>
+      <c r="D187" s="8"/>
+      <c r="E187" s="8"/>
     </row>
     <row r="188">
-      <c r="B188" s="7"/>
-      <c r="C188" s="7"/>
-      <c r="D188" s="7"/>
-      <c r="E188" s="7"/>
+      <c r="B188" s="8"/>
+      <c r="C188" s="8"/>
+      <c r="D188" s="8"/>
+      <c r="E188" s="8"/>
     </row>
     <row r="189">
-      <c r="B189" s="7"/>
-      <c r="C189" s="7"/>
-      <c r="D189" s="7"/>
-      <c r="E189" s="7"/>
+      <c r="B189" s="8"/>
+      <c r="C189" s="8"/>
+      <c r="D189" s="8"/>
+      <c r="E189" s="8"/>
     </row>
     <row r="190">
-      <c r="B190" s="7"/>
-      <c r="C190" s="7"/>
-      <c r="D190" s="7"/>
-      <c r="E190" s="7"/>
+      <c r="B190" s="8"/>
+      <c r="C190" s="8"/>
+      <c r="D190" s="8"/>
+      <c r="E190" s="8"/>
     </row>
     <row r="191">
-      <c r="B191" s="7"/>
-      <c r="C191" s="7"/>
-      <c r="D191" s="7"/>
-      <c r="E191" s="7"/>
+      <c r="B191" s="8"/>
+      <c r="C191" s="8"/>
+      <c r="D191" s="8"/>
+      <c r="E191" s="8"/>
     </row>
     <row r="192">
-      <c r="B192" s="7"/>
-      <c r="C192" s="7"/>
-      <c r="D192" s="7"/>
-      <c r="E192" s="7"/>
+      <c r="B192" s="8"/>
+      <c r="C192" s="8"/>
+      <c r="D192" s="8"/>
+      <c r="E192" s="8"/>
     </row>
     <row r="193">
-      <c r="B193" s="7"/>
-      <c r="C193" s="7"/>
-      <c r="D193" s="7"/>
-      <c r="E193" s="7"/>
+      <c r="B193" s="8"/>
+      <c r="C193" s="8"/>
+      <c r="D193" s="8"/>
+      <c r="E193" s="8"/>
     </row>
     <row r="194">
-      <c r="B194" s="7"/>
-      <c r="C194" s="7"/>
-      <c r="D194" s="7"/>
-      <c r="E194" s="7"/>
+      <c r="B194" s="8"/>
+      <c r="C194" s="8"/>
+      <c r="D194" s="8"/>
+      <c r="E194" s="8"/>
     </row>
     <row r="195">
-      <c r="B195" s="7"/>
-      <c r="C195" s="7"/>
-      <c r="D195" s="7"/>
-      <c r="E195" s="7"/>
+      <c r="B195" s="8"/>
+      <c r="C195" s="8"/>
+      <c r="D195" s="8"/>
+      <c r="E195" s="8"/>
     </row>
     <row r="196">
-      <c r="B196" s="7"/>
-      <c r="C196" s="7"/>
-      <c r="D196" s="7"/>
-      <c r="E196" s="7"/>
+      <c r="B196" s="8"/>
+      <c r="C196" s="8"/>
+      <c r="D196" s="8"/>
+      <c r="E196" s="8"/>
     </row>
     <row r="197">
-      <c r="B197" s="7"/>
-      <c r="C197" s="7"/>
-      <c r="D197" s="7"/>
-      <c r="E197" s="7"/>
+      <c r="B197" s="8"/>
+      <c r="C197" s="8"/>
+      <c r="D197" s="8"/>
+      <c r="E197" s="8"/>
     </row>
     <row r="198">
-      <c r="B198" s="7"/>
-      <c r="C198" s="7"/>
-      <c r="D198" s="7"/>
-      <c r="E198" s="7"/>
+      <c r="B198" s="8"/>
+      <c r="C198" s="8"/>
+      <c r="D198" s="8"/>
+      <c r="E198" s="8"/>
     </row>
     <row r="199">
-      <c r="B199" s="7"/>
-      <c r="C199" s="7"/>
-      <c r="D199" s="7"/>
-      <c r="E199" s="7"/>
+      <c r="B199" s="8"/>
+      <c r="C199" s="8"/>
+      <c r="D199" s="8"/>
+      <c r="E199" s="8"/>
     </row>
     <row r="200">
-      <c r="B200" s="7"/>
-      <c r="C200" s="7"/>
-      <c r="D200" s="7"/>
-      <c r="E200" s="7"/>
+      <c r="B200" s="8"/>
+      <c r="C200" s="8"/>
+      <c r="D200" s="8"/>
+      <c r="E200" s="8"/>
     </row>
     <row r="201">
-      <c r="B201" s="7"/>
-      <c r="C201" s="7"/>
-      <c r="D201" s="7"/>
-      <c r="E201" s="7"/>
+      <c r="B201" s="8"/>
+      <c r="C201" s="8"/>
+      <c r="D201" s="8"/>
+      <c r="E201" s="8"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>